<commit_message>
Update 7-Excel-Sort in Excel.xlsx
</commit_message>
<xml_diff>
--- a/Lesson 7-Sort Data in Excel/7-Excel-Sort in Excel.xlsx
+++ b/Lesson 7-Sort Data in Excel/7-Excel-Sort in Excel.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\91926\Downloads\SD108\Lesson 7-Sort Data in Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c74d3d6648322357/Documents/GitHub/Excel-Learning/Lesson 7-Sort Data in Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{838D48D1-8600-43D5-939A-B32DF2ACFA05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{838D48D1-8600-43D5-939A-B32DF2ACFA05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CE78F4FA-5C47-41C6-A7F9-436A7F1450BF}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Employee Data" sheetId="1" r:id="rId1"/>
@@ -341,23 +341,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="13">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF7C80"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFF7C80"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill>
@@ -369,77 +353,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFF7C80"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF6390C9"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF6390C9"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF8BADD8"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF8BADD8"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5213,18 +5126,6 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N102">
     <sortCondition ref="A1:A102"/>
   </sortState>
-  <conditionalFormatting sqref="K1:K1048576">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF5A8AC6"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9716,6 +9617,14 @@
     <sortCondition ref="E2:E111" customList="Finance"/>
     <sortCondition descending="1" ref="F2:F111"/>
   </sortState>
+  <conditionalFormatting sqref="E1:E1048576">
+    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Finance">
+      <formula>NOT(ISERROR(SEARCH("Finance",E1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="HR">
+      <formula>NOT(ISERROR(SEARCH("HR",E1)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="K1:K1048576">
     <cfRule type="colorScale" priority="3">
       <colorScale>
@@ -9728,14 +9637,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E1:E1048576">
-    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="HR">
-      <formula>NOT(ISERROR(SEARCH("HR",E1)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Finance">
-      <formula>NOT(ISERROR(SEARCH("Finance",E1)))</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>